<commit_message>
doc: set the language to English.
</commit_message>
<xml_diff>
--- a/Tests/excel/module05_test_cases.xlsx
+++ b/Tests/excel/module05_test_cases.xlsx
@@ -1379,7 +1379,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="165" customHeight="1">
+    <row r="2" ht="180" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>TC-M05-001</t>
@@ -1402,41 +1402,41 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>Tạo nhóm thực tập mới với thông tin hợp lệ</t>
+          <t>Create new internship group voi thong tin hop le</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng tạo nhóm thực tập mới khi nhập đầy đủ các thông tin bắt buộc và hợp lệ.</t>
+          <t>Verify functionality for create new internship group khi enter day du cac thong tin bat buoc va hop le.</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện Quản lý Thực tập.
-Các lớp học "PNV26A" và "PNV26B" đã tồn tại trong hệ thống và chưa được gán vào bất kỳ nhóm thực tập nào trong cùng năm học.</t>
+          <t>User is logged in as Staff.
+Currently on Internship Management interface.
+Cac lop hoc "PNV26A" va "PNV26B" da exist in system va chua duoc gan vao bat ky internship group nao trong cung nam hoc.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm Thực tập 2026 - Năm 2"; InternshipYear="Second Year"; Batches="PNV26A", "PNV26B"; StartDate="2026-08-01"</t>
+          <t>GroupName="Nhom Thuc tap 2026 - Nam 2"; InternshipYear="Second Year"; Batches="PNV26A", "PNV26B"; StartDate="2026-08-01"</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>1. Nhấn nút "Tạo nhóm thực tập mới".
-2. Nhập Tên nhóm là "Nhóm Thực tập 2026 - Năm 2".
-3. Chọn Năm thực tập là "Second Year".
-4. Tích chọn các lớp học "PNV26A" và "PNV26B".
-5. Chọn Ngày bắt đầu là "2026-08-01".
-6. Nhấn nút "Lưu".</t>
+          <t>1. Nhan nut "Create new internship group".
+2. Enter Ten group la "Nhom Thuc tap 2026 - Nam 2".
+3. Select Nam internship la "Second Year".
+4. Tich select cac lop hoc "PNV26A" va "PNV26B".
+5. Select Start Date la "2026-08-01".
+6. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo tạo nhóm thành công.
-Nhóm thực tập mới xuất hiện trong danh sách hiển thị với trạng thái là "On-going".
-Các lớp học đã chọn được liên kết chính xác với nhóm này.</t>
+          <t>System display notification create group successfully.
+Nhom internship moi xuat hien trong danh sach display voi status la "On-going".
+Cac lop hoc da select duoc lien ket chinh xac voi group nay.</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr"/>
@@ -1452,11 +1452,11 @@
       </c>
       <c r="N2" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F01, Rule 6.1</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="120" customHeight="1">
+          <t>Related to M05-F01, Rule 6.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="135" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>TC-M05-002</t>
@@ -1479,19 +1479,19 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>Tạo nhóm thực tập thất bại do để trống tên nhóm</t>
+          <t>Internship group creation fails due to empty group name</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống báo lỗi và ngăn chặn tạo nhóm thực tập nếu để trống tên nhóm.</t>
+          <t>Verify system bao error va ngan chan create internship group neu blank ten group.</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện Tạo nhóm thực tập mới.
-Lớp học "PNV26A" chưa được gán cho nhóm thực tập nào trong năm học.</t>
+          <t>User is logged in as Staff.
+Currently on Create New Internship Group interface.
+Lop hoc "PNV26A" chua duoc gan cho internship group nao trong nam hoc.</t>
         </is>
       </c>
       <c r="H3" s="9" t="inlineStr">
@@ -1501,17 +1501,17 @@
       </c>
       <c r="I3" s="9" t="inlineStr">
         <is>
-          <t>1. Để trống trường Tên nhóm.
-2. Chọn Năm thực tập là "Second Year".
-3. Tích chọn lớp học "PNV26A".
-4. Chọn Ngày bắt đầu là "2026-08-01".
-5. Nhấn nút "Lưu".</t>
+          <t>1. De trong truong Ten group.
+2. Select Nam internship la "Second Year".
+3. Tich select lop hoc "PNV26A".
+4. Select Start Date la "2026-08-01".
+5. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J3" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo lỗi yêu cầu nhập Tên nhóm (ví dụ: "Group Name is required.").
-Nhóm thực tập mới không được lưu vào hệ thống.</t>
+          <t>System display notification error requires enter Ten group (e.g.: "Group Name is required.").
+Nhom internship moi khong duoc save vao system.</t>
         </is>
       </c>
       <c r="K3" s="9" t="inlineStr"/>
@@ -1527,7 +1527,7 @@
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến Validation Rules (Mục 7), Error Handling (Mục 8)</t>
+          <t>Related to Validation Rules (Section 7), Error Handling (Section 8)</t>
         </is>
       </c>
     </row>
@@ -1554,38 +1554,38 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Tạo nhóm thực tập thất bại do không tích chọn lớp học</t>
+          <t>Create internship group failed do khong tich select lop hoc</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống báo lỗi và ngăn chặn tạo nhóm thực tập nếu không chọn bất kỳ lớp học nào.</t>
+          <t>Verify system bao error va ngan chan create internship group neu khong select bat ky lop hoc nao.</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện Tạo nhóm thực tập mới.</t>
+          <t>User is logged in as Staff.
+Currently on Create New Internship Group interface.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm Thực tập 2026"; InternshipYear="Second Year"; Batches=None; StartDate="2026-08-01"</t>
+          <t>GroupName="Nhom Thuc tap 2026"; InternshipYear="Second Year"; Batches=None; StartDate="2026-08-01"</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>1. Nhập Tên nhóm là "Nhóm Thực tập 2026".
-2. Chọn Năm thực tập là "Second Year".
-3. Không chọn bất kỳ lớp học nào trong danh sách.
-4. Chọn Ngày bắt đầu là "2026-08-01".
-5. Nhấn nút "Lưu".</t>
+          <t>1. Enter Ten group la "Nhom Thuc tap 2026".
+2. Select Nam internship la "Second Year".
+3. Khong select bat ky lop hoc nao trong danh sach.
+4. Select Start Date la "2026-08-01".
+5. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo lỗi yêu cầu chọn ít nhất một lớp học (ví dụ: "At least one batch is required.").
-Nhóm thực tập mới không được lưu vào hệ thống.</t>
+          <t>System display notification error requires select it nhat mot lop hoc (e.g.: "At least one batch is required.").
+Nhom internship moi khong duoc save vao system.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr"/>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến Validation Rules (Mục 7), Error Handling (Mục 8)</t>
+          <t>Related to Validation Rules (Section 7), Error Handling (Section 8)</t>
         </is>
       </c>
     </row>
@@ -1628,38 +1628,38 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Tạo nhóm thực tập thất bại do để trống ngày bắt đầu</t>
+          <t>Create internship group failed do blank start date</t>
         </is>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống báo lỗi và ngăn chặn tạo nhóm thực tập nếu để trống ngày bắt đầu.</t>
+          <t>Verify system bao error va ngan chan create internship group neu blank start date.</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện Tạo nhóm thực tập mới.</t>
+          <t>User is logged in as Staff.
+Currently on Create New Internship Group interface.</t>
         </is>
       </c>
       <c r="H5" s="9" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm Thực tập 2026"; InternshipYear="Second Year"; Batches="PNV26A"; StartDate=""</t>
+          <t>GroupName="Nhom Thuc tap 2026"; InternshipYear="Second Year"; Batches="PNV26A"; StartDate=""</t>
         </is>
       </c>
       <c r="I5" s="9" t="inlineStr">
         <is>
-          <t>1. Nhập Tên nhóm là "Nhóm Thực tập 2026".
-2. Chọn Năm thực tập là "Second Year".
-3. Tích chọn lớp học "PNV26A".
-4. Để trống trường Ngày bắt đầu.
-5. Nhấn nút "Lưu".</t>
+          <t>1. Enter Ten group la "Nhom Thuc tap 2026".
+2. Select Nam internship la "Second Year".
+3. Tich select lop hoc "PNV26A".
+4. De trong truong Start Date.
+5. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J5" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo lỗi yêu cầu chọn Ngày bắt đầu (ví dụ: "Start Date is required.").
-Nhóm thực tập mới không được lưu vào hệ thống.</t>
+          <t>System display notification error requires select Start Date (e.g.: "Start Date is required.").
+Nhom internship moi khong duoc save vao system.</t>
         </is>
       </c>
       <c r="K5" s="9" t="inlineStr"/>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="N5" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến Validation Rules (Mục 7), Error Handling (Mục 8)</t>
+          <t>Related to Validation Rules (Section 7), Error Handling (Section 8)</t>
         </is>
       </c>
     </row>
@@ -1702,38 +1702,38 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>Tạo nhóm thực tập thất bại do để trống năm thực tập</t>
+          <t>Create internship group failed do blank nam internship</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống báo lỗi và ngăn chặn tạo nhóm thực tập nếu năm thực tập không được chọn.</t>
+          <t>Verify system bao error va ngan chan create internship group neu nam internship khong duoc select.</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện Tạo nhóm thực tập mới.</t>
+          <t>User is logged in as Staff.
+Currently on Create New Internship Group interface.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm Thực tập 2026"; InternshipYear=""; Batches="PNV26A"; StartDate="2026-08-01"</t>
+          <t>GroupName="Nhom Thuc tap 2026"; InternshipYear=""; Batches="PNV26A"; StartDate="2026-08-01"</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>1. Nhập Tên nhóm là "Nhóm Thực tập 2026".
-2. Không chọn Năm thực tập (để trống).
-3. Tích chọn lớp học "PNV26A".
-4. Chọn Ngày bắt đầu là "2026-08-01".
-5. Nhấn nút "Lưu".</t>
+          <t>1. Enter Ten group la "Nhom Thuc tap 2026".
+2. Khong select Nam internship (blank).
+3. Tich select lop hoc "PNV26A".
+4. Select Start Date la "2026-08-01".
+5. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo lỗi yêu cầu chọn Năm thực tập (ví dụ: "Internship Year is required.").
-Nhóm thực tập mới không được lưu vào hệ thống.</t>
+          <t>System display notification error requires select Nam internship (e.g.: "Internship Year is required.").
+Nhom internship moi khong duoc save vao system.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr"/>
@@ -1749,11 +1749,11 @@
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến Validation Rules (Mục 7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="150" customHeight="1">
+          <t>Related to Validation Rules (Section 7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="165" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>TC-M05-006</t>
@@ -1776,39 +1776,39 @@
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Tạo nhóm thực tập thất bại do chọn lớp học đã được gán vào nhóm thực tập khác trong cùng năm học</t>
+          <t>Create internship group failed do select lop hoc da duoc gan vao internship group khac trong cung nam hoc</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống từ chối tạo nhóm thực tập mới chứa lớp học đã được gán cho nhóm thực tập khác trong cùng năm học.</t>
+          <t>Verify system denies create new internship group chua lop hoc da duoc gan cho internship group khac trong cung nam hoc.</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đã tồn tại nhóm thực tập "Nhóm A" cho năm học "Second Year" chứa lớp "PNV26A".</t>
+          <t>User is logged in as Staff.
+Da ton tai internship group "Nhom A" cho nam hoc "Second Year" chua lop "PNV26A".</t>
         </is>
       </c>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm B"; InternshipYear="Second Year"; Batches="PNV26A"; StartDate="2026-08-01"</t>
+          <t>GroupName="Nhom B"; InternshipYear="Second Year"; Batches="PNV26A"; StartDate="2026-08-01"</t>
         </is>
       </c>
       <c r="I7" s="9" t="inlineStr">
         <is>
-          <t>1. Nhấn nút "Tạo nhóm thực tập mới".
-2. Nhập Tên nhóm là "Nhóm B".
-3. Chọn Năm thực tập là "Second Year".
-4. Chọn lớp học là "PNV26A".
-5. Chọn Ngày bắt đầu là "2026-08-01".
-6. Nhấn nút "Lưu".</t>
+          <t>1. Nhan nut "Create new internship group".
+2. Enter Ten group la "Nhom B".
+3. Select Nam internship la "Second Year".
+4. Select lop hoc la "PNV26A".
+5. Select Start Date la "2026-08-01".
+6. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống từ chối lưu và hiển thị thông báo lỗi (ví dụ: lớp PNV26A đã được gán cho một nhóm thực tập khác trong năm học này - "Batch already assigned").
-Nhóm thực tập "Nhóm B" không được tạo.</t>
+          <t>System denies save va display notification error (e.g.: lop PNV26A da duoc gan cho mot internship group khac trong nam hoc nay - "Batch already assigned").
+Nhom internship "Nhom B" khong duoc create.</t>
         </is>
       </c>
       <c r="K7" s="9" t="inlineStr"/>
@@ -1824,11 +1824,11 @@
       </c>
       <c r="N7" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến Batch Assignment Rule (Rule 6.2), Error Handling (Mục 8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="150" customHeight="1">
+          <t>Related to Batch Assignment Rule (Rule 6.2), Error Handling (Section 8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="165" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>TC-M05-007</t>
@@ -1851,39 +1851,39 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Tạo nhóm thực tập thành công khi gán cùng lớp học vào nhóm thực tập ở các năm học khác nhau</t>
+          <t>Create internship group successfully khi gan cung lop hoc vao internship group o cac nam hoc khac nhau</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống cho phép gán cùng một lớp học vào nhóm thực tập ở các năm khác nhau (ví dụ: năm 2 và năm 3).</t>
+          <t>Verify system allows gan cung mot lop hoc vao internship group o cac nam khac nhau (e.g.: nam 2 va nam 3).</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Lớp "PNV26A" đã được gán vào nhóm thực tập "Nhóm Năm 2" thuộc năm thực tập "Second Year".</t>
+          <t>User is logged in as Staff.
+Lop "PNV26A" da duoc gan vao internship group "Nhom Nam 2" thuoc nam internship "Second Year".</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm Năm 3"; InternshipYear="Third Year"; Batches="PNV26A"; StartDate="2027-08-01"</t>
+          <t>GroupName="Nhom Nam 3"; InternshipYear="Third Year"; Batches="PNV26A"; StartDate="2027-08-01"</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>1. Nhấn nút "Tạo nhóm thực tập mới".
-2. Nhập Tên nhóm là "Nhóm Năm 3".
-3. Chọn Năm thực tập là "Third Year".
-4. Chọn lớp học là "PNV26A".
-5. Chọn Ngày bắt đầu là "2027-08-01".
-6. Nhấn nút "Lưu".</t>
+          <t>1. Nhan nut "Create new internship group".
+2. Enter Ten group la "Nhom Nam 3".
+3. Select Nam internship la "Third Year".
+4. Select lop hoc la "PNV26A".
+5. Select Start Date la "2027-08-01".
+6. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống lưu thành công nhóm thực tập mới.
-Lớp PNV26A được gán vào nhóm "Nhóm Năm 3" mà không có lỗi.</t>
+          <t>System save successfully new internship group.
+Lop PNV26A duoc gan vao group "Nhom Nam 3" ma khong co error.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr"/>
@@ -1899,7 +1899,7 @@
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến Batch Assignment Rule (Rule 6.2)</t>
+          <t>Related to Batch Assignment Rule (Rule 6.2)</t>
         </is>
       </c>
     </row>
@@ -1926,37 +1926,37 @@
       </c>
       <c r="E9" s="9" t="inlineStr">
         <is>
-          <t>Lưu trữ nhóm thực tập đang hoạt động</t>
+          <t>Archive internship group dang hoat dong</t>
         </is>
       </c>
       <c r="F9" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng Lưu trữ (Archive) một nhóm thực tập đang ở trạng thái On-going.</t>
+          <t>Verify functionality for Archive (Archive) mot internship group dang o status On-going.</t>
         </is>
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đã tồn tại nhóm thực tập "Nhóm Thực tập 2026" ở trạng thái On-going.</t>
+          <t>User is logged in as Staff.
+Da ton tai internship group "Nhom Thuc tap 2026" o status On-going.</t>
         </is>
       </c>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm Thực tập 2026"</t>
+          <t>GroupName="Nhom Thuc tap 2026"</t>
         </is>
       </c>
       <c r="I9" s="9" t="inlineStr">
         <is>
-          <t>1. Tìm nhóm thực tập "Nhóm Thực tập 2026" trên giao diện danh sách.
-2. Nhấn vào biểu tượng/nút "Lưu trữ" (Archive) của nhóm này.
-3. Xác nhận lưu trữ ở hộp thoại xác nhận.</t>
+          <t>1. Tim internship group "Nhom Thuc tap 2026" tren interface danh sach.
+2. Nhan vao bieu tuong/nut "Archive" (Archive) cua group nay.
+3. Xac nhan archive o hop thoai xac nhan.</t>
         </is>
       </c>
       <c r="J9" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo lưu trữ thành công.
-Trạng thái của nhóm thực tập chuyển sang "Archived".
-Nhóm thực tập này bị ẩn khỏi danh sách hoạt động bình thường.</t>
+          <t>System display notification archive successfully.
+Status cua internship group chuyen sang "Archived".
+Nhom internship nay bi an khoi danh sach hoat dong binh thuong.</t>
         </is>
       </c>
       <c r="K9" s="9" t="inlineStr"/>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="N9" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F02, Rule 6.12</t>
+          <t>Related to M05-F02, Rule 6.12</t>
         </is>
       </c>
     </row>
@@ -1999,38 +1999,38 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Kích hoạt lại nhóm thực tập đã lưu trữ</t>
+          <t>Kich hoat lai internship group da archive</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng khôi phục/kích hoạt lại (Reactivate) một nhóm thực tập đã bị lưu trữ.</t>
+          <t>Verify functionality for khoi phuc/kich hoat lai (Reactivate) mot internship group da bi archive.</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đã có nhóm thực tập "Nhóm Thực tập 2026" ở trạng thái Archived.</t>
+          <t>User is logged in as Staff.
+Da co internship group "Nhom Thuc tap 2026" o status Archived.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm Thực tập 2026"</t>
+          <t>GroupName="Nhom Thuc tap 2026"</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>1. Truy cập vào danh sách các nhóm thực tập đã lưu trữ (Archived Groups).
-2. Tìm nhóm "Nhóm Thực tập 2026".
-3. Nhấn vào nút "Khôi phục" hoặc "Kích hoạt lại" (Reactivate).
-4. Xác nhận ở hộp thoại.</t>
+          <t>1. Truy cap vao danh sach cac internship group da archive (Archived Groups).
+2. Tim group "Nhom Thuc tap 2026".
+3. Nhan vao nut "Khoi phuc" hoac "Kich hoat lai" (Reactivate).
+4. Xac nhan o hop thoai.</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo kích hoạt lại thành công.
-Trạng thái của nhóm chuyển từ "Archived" về "On-going".
-Nhóm thực tập xuất hiện trở lại trong danh sách nhóm đang hoạt động.</t>
+          <t>System display notification kich hoat lai successfully.
+Status cua group chuyen tu "Archived" ve "On-going".
+Nhom internship xuat hien tro lai trong danh sach group dang hoat dong.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr"/>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F02, Rule 6.12</t>
+          <t>Related to M05-F02, Rule 6.12</t>
         </is>
       </c>
     </row>
@@ -2073,18 +2073,18 @@
       </c>
       <c r="E11" s="9" t="inlineStr">
         <is>
-          <t>Thêm công ty đối tác mới với tên hợp lệ</t>
+          <t>Add company doi tac moi with a valid name</t>
         </is>
       </c>
       <c r="F11" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng thêm mới công ty đối tác với tên hợp lệ và chưa tồn tại.</t>
+          <t>Verify functionality for add moi company doi tac with a valid name va chua ton tai.</t>
         </is>
       </c>
       <c r="G11" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện Quản lý Công ty (Company Management).</t>
+          <t>User is logged in as Staff.
+Dang o interface Quan ly Cong ty (Company Management).</t>
         </is>
       </c>
       <c r="H11" s="9" t="inlineStr">
@@ -2094,15 +2094,15 @@
       </c>
       <c r="I11" s="9" t="inlineStr">
         <is>
-          <t>1. Nhấn nút "Thêm công ty mới".
-2. Nhập vào trường Tên công ty: "TechCorp".
-3. Nhấn nút "Lưu".</t>
+          <t>1. Nhan nut "Add company moi".
+2. Enter vao truong Ten company: "TechCorp".
+3. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J11" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo thêm công ty thành công.
-Công ty "TechCorp" xuất hiện trong danh sách các công ty đối tác.</t>
+          <t>System display notification add company successfully.
+Cong ty "TechCorp" xuat hien trong danh sach cac company doi tac.</t>
         </is>
       </c>
       <c r="K11" s="9" t="inlineStr"/>
@@ -2118,7 +2118,7 @@
       </c>
       <c r="N11" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F03, Rule 6.3</t>
+          <t>Related to M05-F03, Rule 6.3</t>
         </is>
       </c>
     </row>
@@ -2145,18 +2145,18 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>Thêm công ty thất bại do để trống tên công ty</t>
+          <t>Add company failed due to empty name company</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống hiển thị thông báo lỗi và ngăn chặn thêm công ty nếu để trống tên công ty.</t>
+          <t>Verify system display notification error va ngan chan add company neu blank ten company.</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện Quản lý Công ty.</t>
+          <t>User is logged in as Staff.
+Dang o interface Quan ly Cong ty.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
@@ -2166,15 +2166,15 @@
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>1. Nhấn nút "Thêm công ty mới".
-2. Để trống trường Tên công ty.
-3. Nhấn nút "Lưu".</t>
+          <t>1. Nhan nut "Add company moi".
+2. De trong truong Ten company.
+3. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo lỗi yêu cầu nhập tên công ty (ví dụ: "Company Name is required.").
-Công ty mới không được thêm vào danh sách.</t>
+          <t>System display notification error requires enter ten company (e.g.: "Company Name is required.").
+Cong ty moi khong duoc add vao danh sach.</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr"/>
@@ -2190,11 +2190,11 @@
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến Validation Rules (Mục 7), Error Handling (Mục 8)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="90" customHeight="1">
+          <t>Related to Validation Rules (Section 7), Error Handling (Section 8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="75" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>TC-M05-012</t>
@@ -2217,19 +2217,19 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>Thêm công ty thất bại do trùng tên (phân biệt hoa thường)</t>
+          <t>Add company failed do trung ten (phan biet hoa thuong)</t>
         </is>
       </c>
       <c r="F13" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống từ chối và báo lỗi khi thêm công ty có tên viết hoa/thường trùng với công ty đã tồn tại.</t>
+          <t>Verify system denies va bao error khi add company co ten viet hoa/thuong trung voi company da ton tai.</t>
         </is>
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đã tồn tại công ty "TechCorp" trong hệ thống.
-Đang ở giao diện Quản lý Công ty.</t>
+          <t>User is logged in as Staff.
+Da ton tai company "TechCorp" trong system.
+Dang o interface Quan ly Cong ty.</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
@@ -2239,15 +2239,15 @@
       </c>
       <c r="I13" s="9" t="inlineStr">
         <is>
-          <t>1. Nhấn nút "Thêm công ty mới".
-2. Nhập vào trường Tên công ty: "techcorp" (viết thường hoàn toàn).
-3. Nhấn nút "Lưu".</t>
+          <t>1. Nhan nut "Add company moi".
+2. Enter vao truong Ten company: "techcorp" (viet thuong hoan toan).
+3. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống từ chối lưu và hiển thị thông báo lỗi trùng tên công ty (ví dụ: "Company name already exists.").
-Công ty trùng lặp không được tạo thêm.</t>
+          <t>System denies save va display notification error trung ten company (e.g.: "Company name already exists.").
+Cong ty trung lap khong duoc create add.</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr"/>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="N13" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F03, Rule 6.3, Error Handling (Mục 8)</t>
+          <t>Related to M05-F03, Rule 6.3, Error Handling (Section 8)</t>
         </is>
       </c>
     </row>
@@ -2290,36 +2290,36 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Thêm công ty thất bại do trùng tên khi có khoảng trắng đầu/cuối</t>
+          <t>Add company failed do trung ten khi co khoang trang dau/cuoi</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống tự động loại bỏ khoảng trắng đầu/cuối và từ chối nếu tên công ty trùng lặp.</t>
+          <t>Verify system tu dong loai bo khoang trang dau/cuoi va denies neu ten company trung lap.</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đã tồn tại công ty "TechCorp" trong hệ thống.
-Đang ở giao diện Quản lý Công ty.</t>
+          <t>User is logged in as Staff.
+Da ton tai company "TechCorp" trong system.
+Dang o interface Quan ly Cong ty.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>CompanyName="  TechCorp  "</t>
+          <t>CompanyName=" TechCorp "</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>1. Nhấn nút "Thêm công ty mới".
-2. Nhập vào trường Tên công ty: "  TechCorp  " (có khoảng trắng ở đầu và cuối).
-3. Nhấn nút "Lưu".</t>
+          <t>1. Nhan nut "Add company moi".
+2. Enter vao truong Ten company: " TechCorp " (co khoang trang o dau va cuoi).
+3. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống cắt bỏ các khoảng trắng đầu/cuối, phát hiện trùng lặp với "TechCorp", từ chối lưu và hiển thị thông báo lỗi trùng tên.</t>
+          <t>System cat bo cac khoang trang dau/cuoi, phat hien trung lap voi "TechCorp", denies save va display notification error trung ten.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr"/>
@@ -2335,7 +2335,7 @@
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F03, Rule 6.3, Error Handling (Mục 8)</t>
+          <t>Related to M05-F03, Rule 6.3, Error Handling (Section 8)</t>
         </is>
       </c>
     </row>
@@ -2362,40 +2362,40 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Phân công thực tập cho học viên đơn lẻ</t>
+          <t>Phan cong internship cho student don le</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng phân công một học viên vào một công ty đối tác.</t>
+          <t>Verify functionality for phan cong mot student vao mot company doi tac.</t>
         </is>
       </c>
       <c r="G15" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện danh sách học viên của nhóm thực tập "Nhóm Thực tập 2026" (trạng thái On-going).
-Học viên "Nguyễn Văn A" đang ở trạng thái chưa được phân công (Unassigned).
-Công ty "TechCorp" đang ở trạng thái hoạt động (không bị ẩn).</t>
+          <t>User is logged in as Staff.
+Dang o interface danh sach student cua internship group "Nhom Thuc tap 2026" (status On-going).
+Hoc vien "Nguyen Van A" dang o status chua duoc phan cong (Unassigned).
+Cong ty "TechCorp" dang o status hoat dong (khong bi an).</t>
         </is>
       </c>
       <c r="H15" s="9" t="inlineStr">
         <is>
-          <t>StudentName="Nguyễn Văn A"; AssignedCompany="TechCorp"</t>
+          <t>StudentName="Nguyen Van A"; AssignedCompany="TechCorp"</t>
         </is>
       </c>
       <c r="I15" s="9" t="inlineStr">
         <is>
-          <t>1. Tìm học viên "Nguyễn Văn A" trong bảng phân công học viên.
-2. Nhấp vào ô chọn công ty của học viên "Nguyễn Văn A".
-3. Chọn công ty "TechCorp" từ danh sách gợi ý.
-4. Nhấn nút "Lưu thay đổi".</t>
+          <t>1. Tim student "Nguyen Van A" trong bang phan cong student.
+2. Nhap vao o select company cua student "Nguyen Van A".
+3. Select company "TechCorp" tu danh sach goi y.
+4. Nhan nut "Save thay doi".</t>
         </is>
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo phân công thành công.
-Học viên "Nguyễn Văn A" hiển thị công ty đã gán là "TechCorp".
-Số lượng học viên chưa phân công trên nhãn cảnh báo (Warning Badge) tự động giảm đi 1.</t>
+          <t>System display notification phan cong successfully.
+Hoc vien "Nguyen Van A" display company da gan la "TechCorp".
+So luong student chua phan cong tren nhan cphoto bao (Warning Badge) tu dong giam di 1.</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr"/>
@@ -2411,11 +2411,11 @@
       </c>
       <c r="N15" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F04, M05-F06, Rule 6.4, Rule 6.11</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="135" customHeight="1">
+          <t>Related to M05-F04, M05-F06, Rule 6.4, Rule 6.11</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="150" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>TC-M05-015</t>
@@ -2438,40 +2438,40 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Phân công thực tập hàng loạt cho nhiều học viên cùng lúc</t>
+          <t>Phan cong internship hang loat cho nhieu student cung luc</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng chọn nhiều học viên và phân công vào cùng một công ty cùng lúc.</t>
+          <t>Verify functionality for select nhieu student va phan cong vao cung mot company cung luc.</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện danh sách học viên của nhóm thực tập.
-Có ít nhất 3 học viên đang ở trạng thái chưa phân công (ví dụ: Nguyễn Văn B, Trần Thị C, Lê Văn D).
-Công ty "TechCorp" đang hoạt động.</t>
+          <t>User is logged in as Staff.
+Dang o interface danh sach student cua internship group.
+Co it nhat 3 student dang o status chua phan cong (e.g.: Nguyen Van B, Tran Thi C, Le Van D).
+Cong ty "TechCorp" dang hoat dong.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>SelectedStudents="Nguyễn Văn B", "Trần Thị C", "Lê Văn D"; AssignedCompany="TechCorp"</t>
+          <t>SelectedStudents="Nguyen Van B", "Tran Thi C", "Le Van D"; AssignedCompany="TechCorp"</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>1. Tích chọn các ô vuông (checkbox) đầu dòng của học viên "Nguyễn Văn B", "Trần Thị C" và "Lê Văn D".
-2. Nhấn nút "Phân công hàng loạt" (Bulk Assign).
-3. Chọn công ty "TechCorp" trong hộp thoại hiện ra.
-4. Nhấn nút "Áp dụng" hoặc "Lưu".</t>
+          <t>1. Tich select cac o vuong (checkbox) dau dong cua student "Nguyen Van B", "Tran Thi C" va "Le Van D".
+2. Nhan nut "Phan cong hang loat" (Bulk Assign).
+3. Select company "TechCorp" trong hop thoai hien ra.
+4. Nhan nut "Ap dung" hoac "Save".</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống hiển thị thông báo phân công hàng loạt thành công.
-Cả 3 học viên trên đều hiển thị công ty được phân công là "TechCorp".
-Số lượng trên nhãn cảnh báo học viên chưa phân công tự động giảm đi 3.</t>
+          <t>System display notification phan cong hang loat successfully.
+Ca 3 student tren deu display company duoc phan cong la "TechCorp".
+So luong tren nhan cphoto bao student chua phan cong tu dong giam di 3.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr"/>
@@ -2487,7 +2487,7 @@
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F04, M05-F06, Rule 6.4, Rule 6.11</t>
+          <t>Related to M05-F04, M05-F06, Rule 6.4, Rule 6.11</t>
         </is>
       </c>
     </row>
@@ -2514,39 +2514,39 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>Thay đổi công ty đã phân công của học viên</t>
+          <t>Thay doi company da phan cong cua student</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng gán công ty mới cho học viên đã được phân công trước đó, đảm bảo công ty cũ bị ghi đè.</t>
+          <t>Verify functionality for gan company moi cho student da duoc phan cong truoc do, dam bao company cu bi ghi de.</t>
         </is>
       </c>
       <c r="G17" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Học viên "Nguyễn Văn A" đang được phân công ở công ty "TechCorp".
-Công ty "PNV Software" đang hoạt động trong hệ thống.</t>
+          <t>User is logged in as Staff.
+Hoc vien "Nguyen Van A" dang duoc phan cong o company "TechCorp".
+Cong ty "PNV Software" dang hoat dong trong system.</t>
         </is>
       </c>
       <c r="H17" s="9" t="inlineStr">
         <is>
-          <t>StudentName="Nguyễn Văn A"; NewCompany="PNV Software"</t>
+          <t>StudentName="Nguyen Van A"; NewCompany="PNV Software"</t>
         </is>
       </c>
       <c r="I17" s="9" t="inlineStr">
         <is>
-          <t>1. Tìm học viên "Nguyễn Văn A" trong danh sách.
-2. Mở danh sách chọn công ty của học viên này và đổi từ "TechCorp" sang "PNV Software".
-3. Nhấn nút "Lưu thay đổi".</t>
+          <t>1. Tim student "Nguyen Van A" trong danh sach.
+2. Mo danh sach select company cua student nay va doi tu "TechCorp" sang "PNV Software".
+3. Nhan nut "Save thay doi".</t>
         </is>
       </c>
       <c r="J17" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống cập nhật thành công.
-Công ty phân công mới của học viên "Nguyễn Văn A" hiển thị là "PNV Software".
-Phân công cũ tại "TechCorp" bị thay thế hoàn toàn.
-Nhãn cảnh báo học viên chưa phân công không thay đổi số lượng.</t>
+          <t>System cap nhat successfully.
+Cong ty phan cong moi cua student "Nguyen Van A" display la "PNV Software".
+Phan cong cu tai "TechCorp" bi replace hoan toan.
+Nhan cphoto bao student chua phan cong khong thay doi so luong.</t>
         </is>
       </c>
       <c r="K17" s="9" t="inlineStr"/>
@@ -2562,7 +2562,7 @@
       </c>
       <c r="N17" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F04, Rule 6.4</t>
+          <t>Related to M05-F04, Rule 6.4</t>
         </is>
       </c>
     </row>
@@ -2589,37 +2589,37 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>Hủy bỏ phân công công ty của học viên bằng cách chọn No Company</t>
+          <t>Huy bo phan cong company cua student bang cach select No Company</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng đưa học viên đã phân công về lại trạng thái chưa phân công (Unassigned) bằng cách chọn "(No Company)".</t>
+          <t>Verify functionality for dua student da phan cong ve lai status chua phan cong (Unassigned) bang cach select "(No Company)".</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Học viên "Nguyễn Văn A" đang được phân công tại công ty "PNV Software".</t>
+          <t>User is logged in as Staff.
+Hoc vien "Nguyen Van A" dang duoc phan cong tai company "PNV Software".</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>StudentName="Nguyễn Văn A"; Selection="(No Company)"</t>
+          <t>StudentName="Nguyen Van A"; Selection="(No Company)"</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>1. Tìm học viên "Nguyễn Văn A" trong danh sách.
-2. Nhấp vào ô chọn công ty, chọn giá trị "(No Company)".
-3. Nhấn nút "Lưu".</t>
+          <t>1. Tim student "Nguyen Van A" trong danh sach.
+2. Nhap vao o select company, select gia tri "(No Company)".
+3. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống lưu thành công.
-Học viên "Nguyễn Văn A" hiển thị trạng thái là chưa được phân công.
-Số lượng trên nhãn cảnh báo học viên chưa phân công (Warning Badge) tự động tăng lên 1.</t>
+          <t>System save successfully.
+Hoc vien "Nguyen Van A" display status la chua duoc phan cong.
+So luong tren nhan cphoto bao student chua phan cong (Warning Badge) tu dong tang len 1.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr"/>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F05, M05-F06, Rule 6.5, Rule 6.11, Error Handling (Mục 8)</t>
+          <t>Related to M05-F05, M05-F06, Rule 6.5, Rule 6.11, Error Handling (Section 8)</t>
         </is>
       </c>
     </row>
@@ -2662,18 +2662,18 @@
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>Ẩn công ty và kiểm tra xem công ty đó có bị loại khỏi danh sách chọn phân công mới hay không</t>
+          <t>An company va kiem tra xem company do co bi loai khoi danh sach select phan cong moi hay khong</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra quy tắc công ty bị ẩn (Hidden) không xuất hiện trong dropdown phân công thực tập mới.</t>
+          <t>Verify quy tac company bi an (Hidden) khong xuat hien trong dropdown phan cong internship moi.</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đã tồn tại công ty "ABC Technology" trong hệ thống.</t>
+          <t>User is logged in as Staff.
+Da ton tai company "ABC Technology" trong system.</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
@@ -2683,16 +2683,16 @@
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>1. Vào trang Quản lý Công ty (Company Management).
-2. Tìm công ty "ABC Technology" và chọn thiết lập "Ẩn" (Hidden) cho công ty này.
-3. Nhấn nút "Lưu trạng thái công ty".
-4. Quay lại trang danh sách học viên của nhóm thực tập và mở dropdown phân công công ty của một học viên bất kỳ chưa được phân công.</t>
+          <t>1. Vao trang Quan ly Cong ty (Company Management).
+2. Tim company "ABC Technology" va select thiet lap "An" (Hidden) cho company nay.
+3. Nhan nut "Save status company".
+4. Quay lai trang danh sach student cua internship group va mo dropdown phan cong company cua mot student bat ky chua duoc phan cong.</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>Trạng thái ẩn được lưu thành công.
-Công ty "ABC Technology" không xuất hiện trong danh sách dropdown để chọn phân công mới.</t>
+          <t>Status an duoc save successfully.
+Cong ty "ABC Technology" khong xuat hien trong danh sach dropdown de select phan cong moi.</t>
         </is>
       </c>
       <c r="K19" s="9" t="inlineStr"/>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="N19" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến Rule 6.6, Error Handling (Mục 8)</t>
+          <t>Related to Rule 6.6, Error Handling (Section 8)</t>
         </is>
       </c>
     </row>
@@ -2735,18 +2735,18 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>Đảm bảo phân công hiện tại của học viên không bị ảnh hưởng khi công ty đó bị ẩn</t>
+          <t>Dam bao phan cong hien tai cua student khong bi photo huong khi company do bi an</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra quy tắc các phân công hiện tại vẫn hiển thị chính xác tên công ty sau khi công ty đó bị chuyển sang ẩn.</t>
+          <t>Verify quy tac cac phan cong hien tai van display chinh xac ten company sau khi company do bi chuyen sang an.</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Học viên "Trần Thị B" đã được phân công tại công ty "ABC Technology".</t>
+          <t>User is logged in as Staff.
+Hoc vien "Tran Thi B" da duoc phan cong tai company "ABC Technology".</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
@@ -2756,15 +2756,15 @@
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>1. Vào trang Quản lý Công ty, chuyển trạng thái của "ABC Technology" sang "Ẩn" (Hidden) và lưu lại.
-2. Đi tới trang danh sách học viên của nhóm thực tập.
-3. Quan sát bản ghi phân công của học viên "Trần Thị B".</t>
+          <t>1. Vao trang Quan ly Cong ty, chuyen status cua "ABC Technology" sang "An" (Hidden) va save lai.
+2. Di toi trang danh sach student cua internship group.
+3. Observe ban ghi phan cong cua student "Tran Thi B".</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Phân công của học viên "Trần Thị B" vẫn được hiển thị là "ABC Technology" một cách bình thường trên giao diện.
-Không có thông báo lỗi hay tự động xóa phân công.</t>
+          <t>Phan cong cua student "Tran Thi B" van duoc display la "ABC Technology" mot cach binh thuong tren interface.
+Khong co notification error hay tu dong delete phan cong.</t>
         </is>
       </c>
       <c r="K20" s="4" t="inlineStr"/>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến Rule 6.6</t>
+          <t>Related to Rule 6.6</t>
         </is>
       </c>
     </row>
@@ -2807,40 +2807,40 @@
       </c>
       <c r="E21" s="9" t="inlineStr">
         <is>
-          <t>Ghi nhận nhận xét thực tập thành công cho một học viên với team Training</t>
+          <t>Ghi nhan nhan xet internship successfully cho mot student voi team Training</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng ghi nhận nhận xét thực tập cho học viên thuộc đội ngũ Training.</t>
+          <t>Verify functionality for ghi nhan nhan xet internship cho student thuoc doi ngu Training.</t>
         </is>
       </c>
       <c r="G21" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện danh sách học viên nhóm thực tập.
-Học viên "Nguyễn Văn A" đã được phân công thực tập.</t>
+          <t>User is logged in as Staff.
+Dang o interface danh sach student internship group.
+Hoc vien "Nguyen Van A" da duoc phan cong internship.</t>
         </is>
       </c>
       <c r="H21" s="9" t="inlineStr">
         <is>
-          <t>StudentName="Nguyễn Văn A"; FeedbackTeam="Training"; FeedbackDate="2026-08-15"; FeedbackNotes="Tiến bộ tốt, chủ động trong công việc."</t>
+          <t>StudentName="Nguyen Van A"; FeedbackTeam="Training"; FeedbackDate="2026-08-15"; FeedbackNotes="Tien bo tot, chu dong trong task."</t>
         </is>
       </c>
       <c r="I21" s="9" t="inlineStr">
         <is>
-          <t>1. Tìm học viên "Nguyễn Văn A" trong danh sách.
-2. Nhấp vào nút "Thêm nhận xét" (Add Feedback) của học viên này.
-3. Chọn Team nhận xét là "Training".
-4. Nhập Ngày nhận xét là "2026-08-15".
-5. Nhập Nội dung nhận xét là "Tiến bộ tốt, chủ động trong công việc.".
-6. Nhấn nút "Lưu nhận xét".</t>
+          <t>1. Tim student "Nguyen Van A" trong danh sach.
+2. Nhap vao nut "Add nhan xet" (Add Feedback) cua student nay.
+3. Select Team nhan xet la "Training".
+4. Enter Ngay nhan xet la "2026-08-15".
+5. Enter Noi dung nhan xet la "Tien bo tot, chu dong trong task.".
+6. Nhan nut "Save nhan xet".</t>
         </is>
       </c>
       <c r="J21" s="9" t="inlineStr">
         <is>
-          <t>Nhận xét được lưu thành công.
-Thông tin nhận xét mới xuất hiện dưới tên học viên với đúng Team "Training", ngày và nội dung nhận xét tương ứng.</t>
+          <t>Nhan xet duoc save successfully.
+Thong tin nhan xet moi xuat hien duoi ten student voi dung Team "Training", ngay va noi dung nhan xet tuong ung.</t>
         </is>
       </c>
       <c r="K21" s="9" t="inlineStr"/>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="N21" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F07, Rule 6.7</t>
+          <t>Related to M05-F07, Rule 6.7</t>
         </is>
       </c>
     </row>
@@ -2883,40 +2883,40 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Ghi nhận nhận xét thực tập thành công cho một học viên với team ERO</t>
+          <t>Ghi nhan nhan xet internship successfully cho mot student voi team ERO</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng ghi nhận nhận xét thực tập cho học viên thuộc đội ngũ ERO.</t>
+          <t>Verify functionality for ghi nhan nhan xet internship cho student thuoc doi ngu ERO.</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện danh sách học viên nhóm thực tập.
-Học viên "Nguyễn Văn A" đã được phân công thực tập.</t>
+          <t>User is logged in as Staff.
+Dang o interface danh sach student internship group.
+Hoc vien "Nguyen Van A" da duoc phan cong internship.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>StudentName="Nguyễn Văn A"; FeedbackTeam="ERO"; FeedbackDate="2026-08-15"; FeedbackNotes="Kỹ năng kỹ thuật tốt, thái độ chuyên nghiệp."</t>
+          <t>StudentName="Nguyen Van A"; FeedbackTeam="ERO"; FeedbackDate="2026-08-15"; FeedbackNotes="Ky nang ky thuat tot, thai do chuyen nghiep."</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
         <is>
-          <t>1. Tìm học viên "Nguyễn Văn A" trong danh sách.
-2. Nhấp vào nút "Thêm nhận xét" (Add Feedback) của học viên này.
-3. Chọn Team nhận xét là "ERO".
-4. Nhập Ngày nhận xét là "2026-08-15".
-5. Nhập Nội dung nhận xét là "Kỹ năng kỹ thuật tốt, thái độ chuyên nghiệp.".
-6. Nhấn nút "Lưu nhận xét".</t>
+          <t>1. Tim student "Nguyen Van A" trong danh sach.
+2. Nhap vao nut "Add nhan xet" (Add Feedback) cua student nay.
+3. Select Team nhan xet la "ERO".
+4. Enter Ngay nhan xet la "2026-08-15".
+5. Enter Noi dung nhan xet la "Ky nang ky thuat tot, thai do chuyen nghiep.".
+6. Nhan nut "Save nhan xet".</t>
         </is>
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>Nhận xét được lưu thành công.
-Thông tin nhận xét mới xuất hiện dưới tên học viên với đúng Team "ERO", ngày và nội dung nhận xét tương ứng.</t>
+          <t>Nhan xet duoc save successfully.
+Thong tin nhan xet moi xuat hien duoi ten student voi dung Team "ERO", ngay va noi dung nhan xet tuong ung.</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr"/>
@@ -2932,7 +2932,7 @@
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F07, Rule 6.7</t>
+          <t>Related to M05-F07, Rule 6.7</t>
         </is>
       </c>
     </row>
@@ -2959,40 +2959,40 @@
       </c>
       <c r="E23" s="9" t="inlineStr">
         <is>
-          <t>Ghi nhận nhận xét thực tập thành công cho một học viên với team Educators</t>
+          <t>Ghi nhan nhan xet internship successfully cho mot student voi team Educators</t>
         </is>
       </c>
       <c r="F23" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng ghi nhận nhận xét thực tập cho học viên thuộc đội ngũ Educators.</t>
+          <t>Verify functionality for ghi nhan nhan xet internship cho student thuoc doi ngu Educators.</t>
         </is>
       </c>
       <c r="G23" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện danh sách học viên nhóm thực tập.
-Học viên "Nguyễn Văn A" đã được phân công thực tập.</t>
+          <t>User is logged in as Staff.
+Dang o interface danh sach student internship group.
+Hoc vien "Nguyen Van A" da duoc phan cong internship.</t>
         </is>
       </c>
       <c r="H23" s="9" t="inlineStr">
         <is>
-          <t>StudentName="Nguyễn Văn A"; FeedbackTeam="Educators"; FeedbackDate="2026-08-15"; FeedbackNotes="Năng nổ đóng góp ý kiến xây dựng nhóm."</t>
+          <t>StudentName="Nguyen Van A"; FeedbackTeam="Educators"; FeedbackDate="2026-08-15"; FeedbackNotes="Nang no dong gop y kien xay dung group."</t>
         </is>
       </c>
       <c r="I23" s="9" t="inlineStr">
         <is>
-          <t>1. Tìm học viên "Nguyễn Văn A" trong danh sách.
-2. Nhấp vào nút "Thêm nhận xét" (Add Feedback) của học viên này.
-3. Chọn Team nhận xét là "Educators".
-4. Nhập Ngày nhận xét là "2026-08-15".
-5. Nhập Nội dung nhận xét là "Năng nổ đóng góp ý kiến xây dựng nhóm.".
-6. Nhấn nút "Lưu nhận xét".</t>
+          <t>1. Tim student "Nguyen Van A" trong danh sach.
+2. Nhap vao nut "Add nhan xet" (Add Feedback) cua student nay.
+3. Select Team nhan xet la "Educators".
+4. Enter Ngay nhan xet la "2026-08-15".
+5. Enter Noi dung nhan xet la "Nang no dong gop y kien xay dung group.".
+6. Nhan nut "Save nhan xet".</t>
         </is>
       </c>
       <c r="J23" s="9" t="inlineStr">
         <is>
-          <t>Nhận xét được lưu thành công.
-Thông tin nhận xét mới xuất hiện dưới tên học viên với đúng Team "Educators", ngày và nội dung nhận xét tương ứng.</t>
+          <t>Nhan xet duoc save successfully.
+Thong tin nhan xet moi xuat hien duoi ten student voi dung Team "Educators", ngay va noi dung nhan xet tuong ung.</t>
         </is>
       </c>
       <c r="K23" s="9" t="inlineStr"/>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="N23" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F07, Rule 6.7</t>
+          <t>Related to M05-F07, Rule 6.7</t>
         </is>
       </c>
     </row>
@@ -3035,18 +3035,18 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Bỏ qua các dòng nhận xét trống không lưu vào hệ thống</t>
+          <t>Bo qua cac dong nhan xet trong khong save vao system</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra hệ thống bỏ qua và không lưu các dòng nhận xét không chứa nội dung (trống).</t>
+          <t>Verify system bo qua va khong save cac dong nhan xet khong chua noi dung (trong).</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện Thêm nhận xét cho học viên.</t>
+          <t>User is logged in as Staff.
+Dang o interface Add nhan xet cho student.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
@@ -3056,16 +3056,16 @@
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>1. Mở giao diện nhập nhận xét của học viên.
-2. Chọn Team là "ERO" và chọn ngày nhận xét.
-3. Bỏ trống trường Nội dung nhận xét (Notes).
-4. Nhấn nút "Lưu".</t>
+          <t>1. Mo interface enter nhan xet cua student.
+2. Select Team la "ERO" va select ngay nhan xet.
+3. Bo trong truong Noi dung nhan xet (Notes).
+4. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>Hệ thống bỏ qua dòng nhận xét này, không tạo bản ghi mới trong cơ sở dữ liệu (Google Sheets).
-Không hiển thị thông báo lỗi nhưng cũng không hiển thị bản ghi nhận xét trống này trên UI.</t>
+          <t>System bo qua dong nhan xet nay, khong create ban ghi moi trong co so du lieu (Google Sheets).
+Khong display notification error nhung cung not displayed ban ghi nhan xet trong nay tren UI.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr"/>
@@ -3081,7 +3081,7 @@
       </c>
       <c r="N24" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến Rule 6.8, Error Handling (Mục 8)</t>
+          <t>Related to Rule 6.8, Error Handling (Section 8)</t>
         </is>
       </c>
     </row>
@@ -3108,38 +3108,38 @@
       </c>
       <c r="E25" s="9" t="inlineStr">
         <is>
-          <t>Ghi nhận nhận xét giống nhau cho nhiều học viên cùng lúc (Same for All)</t>
+          <t>Ghi nhan nhan xet giong nhau cho nhieu student cung luc (Same for All)</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra tính năng ghi nhận nhận xét hàng loạt và áp dụng nội dung giống nhau cho các học viên được chọn.</t>
+          <t>Verify tinh nang ghi nhan nhan xet hang loat va ap dung noi dung giong nhau cho cac student duoc select.</t>
         </is>
       </c>
       <c r="G25" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở giao diện danh sách học viên của nhóm thực tập.
-Có ít nhất 2 học viên được chọn (ví dụ: Nguyễn Văn A, Trần Thị B).</t>
+          <t>User is logged in as Staff.
+Dang o interface danh sach student cua internship group.
+Co it nhat 2 student duoc select (e.g.: Nguyen Van A, Tran Thi B).</t>
         </is>
       </c>
       <c r="H25" s="9" t="inlineStr">
         <is>
-          <t>SelectedStudents="Nguyễn Văn A", "Trần Thị B"; FeedbackTeam="Educators"; FeedbackDate="2026-08-15"; FeedbackNotes="Kỹ năng giao tiếp xuất sắc."</t>
+          <t>SelectedStudents="Nguyen Van A", "Tran Thi B"; FeedbackTeam="Educators"; FeedbackDate="2026-08-15"; FeedbackNotes="Ky nang giao tiep xuat sac."</t>
         </is>
       </c>
       <c r="I25" s="9" t="inlineStr">
         <is>
-          <t>1. Tích chọn checkbox của học viên "Nguyễn Văn A" và "Trần Thị B".
-2. Nhấn nút "Nhận xét hàng loạt" (Batch Feedback / Same for All).
-3. Chọn Team là "Educators", chọn Ngày nhận xét là "2026-08-15", nhập Nội dung nhận xét chung là "Kỹ năng giao tiếp xuất sắc.".
-4. Nhấn nút "Áp dụng và Lưu".</t>
+          <t>1. Tich select checkbox cua student "Nguyen Van A" va "Tran Thi B".
+2. Nhan nut "Nhan xet hang loat" (Batch Feedback / Same for All).
+3. Select Team la "Educators", select Ngay nhan xet la "2026-08-15", enter Noi dung nhan xet chung la "Ky nang giao tiep xuat sac.".
+4. Nhan nut "Ap dung va Save".</t>
         </is>
       </c>
       <c r="J25" s="9" t="inlineStr">
         <is>
-          <t>Hệ thống lưu thành công nhận xét cho cả hai học viên.
-Cả học viên "Nguyễn Văn A" và "Trần Thị B" đều hiển thị bản ghi nhận xét của Educators với cùng nội dung "Kỹ năng giao tiếp xuất sắc." vào ngày 2026-08-15.</t>
+          <t>System save successfully nhan xet cho ca hai student.
+Ca student "Nguyen Van A" va "Tran Thi B" deu display ban ghi nhan xet cua Educators voi cung noi dung "Ky nang giao tiep xuat sac." vao ngay 2026-08-15.</t>
         </is>
       </c>
       <c r="K25" s="9" t="inlineStr"/>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="N25" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F08, Rule 6.9</t>
+          <t>Related to M05-F08, Rule 6.9</t>
         </is>
       </c>
     </row>
@@ -3182,37 +3182,37 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>Chỉnh sửa nhận xét thực tập đã lưu (thay đổi nội dung nhận xét)</t>
+          <t>Edit nhan xet internship da save (thay doi noi dung nhan xet)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng chỉnh sửa và lưu đè nội dung nhận xét đã tồn tại.</t>
+          <t>Verify functionality for edit va save de noi dung nhan xet da ton tai.</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Học viên "Nguyễn Văn A" đã có nhận xét: Team = "Training", nội dung = "Tiến bộ tốt", ngày = "2026-08-15".</t>
+          <t>User is logged in as Staff.
+Hoc vien "Nguyen Van A" da co nhan xet: Team = "Training", noi dung = "Tien bo tot", ngay = "2026-08-15".</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>StudentName="Nguyễn Văn A"; NewFeedbackNotes="Tiến bộ vượt bậc và làm việc nhóm tốt."</t>
+          <t>StudentName="Nguyen Van A"; NewFeedbackNotes="Tien bo vuot bac va lam viec group tot."</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>1. Tìm học viên "Nguyễn Văn A" và mở danh sách nhận xét của học viên.
-2. Chọn nhận xét có nội dung "Tiến bộ tốt" và nhấn nút "Chỉnh sửa" (Edit).
-3. Cập nhật nội dung nhận xét thành "Tiến bộ vượt bậc và làm việc nhóm tốt.".
-4. Nhấn nút "Lưu".</t>
+          <t>1. Tim student "Nguyen Van A" va mo danh sach nhan xet cua student.
+2. Select nhan xet co noi dung "Tien bo tot" va click button "Edit" (Edit).
+3. Cap nhat noi dung nhan xet thanh "Tien bo vuot bac va lam viec group tot.".
+4. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>Nhận xét được cập nhật thành công.
-Nội dung mới ghi đè lên nội dung cũ và hiển thị chính xác trên UI: "Tiến bộ vượt bậc và làm việc nhóm tốt.".</t>
+          <t>Nhan xet duoc cap nhat successfully.
+Noi dung moi ghi de len noi dung cu va display chinh xac tren UI: "Tien bo vuot bac va lam viec group tot.".</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr"/>
@@ -3228,7 +3228,7 @@
       </c>
       <c r="N26" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F09, Rule 6.10</t>
+          <t>Related to M05-F09, Rule 6.10</t>
         </is>
       </c>
     </row>
@@ -3255,38 +3255,38 @@
       </c>
       <c r="E27" s="9" t="inlineStr">
         <is>
-          <t>Chỉnh sửa nhận xét thực tập đã lưu (thay đổi team nhận xét và ngày nhận xét)</t>
+          <t>Edit nhan xet internship da save (thay doi team nhan xet va ngay nhan xet)</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng chỉnh sửa và lưu đè thông tin team và ngày nhận xét đã tồn tại.</t>
+          <t>Verify functionality for edit va save de thong tin team va ngay nhan xet da ton tai.</t>
         </is>
       </c>
       <c r="G27" s="9" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Học viên "Nguyễn Văn A" đã có nhận xét: Team = "Training", nội dung = "Tiến bộ tốt", ngày = "2026-08-15".</t>
+          <t>User is logged in as Staff.
+Hoc vien "Nguyen Van A" da co nhan xet: Team = "Training", noi dung = "Tien bo tot", ngay = "2026-08-15".</t>
         </is>
       </c>
       <c r="H27" s="9" t="inlineStr">
         <is>
-          <t>StudentName="Nguyễn Văn A"; NewFeedbackTeam="ERO"; NewFeedbackDate="2026-08-20"</t>
+          <t>StudentName="Nguyen Van A"; NewFeedbackTeam="ERO"; NewFeedbackDate="2026-08-20"</t>
         </is>
       </c>
       <c r="I27" s="9" t="inlineStr">
         <is>
-          <t>1. Tìm học viên "Nguyễn Văn A" và mở danh sách nhận xét của học viên.
-2. Chọn nhận xét có nội dung "Tiến bộ tốt" và nhấn nút "Chỉnh sửa" (Edit).
-3. Thay đổi Team nhận xét thành "ERO".
-4. Thay đổi Ngày nhận xét thành "2026-08-20".
-5. Nhấn nút "Lưu".</t>
+          <t>1. Tim student "Nguyen Van A" va mo danh sach nhan xet cua student.
+2. Select nhan xet co noi dung "Tien bo tot" va click button "Edit" (Edit).
+3. Thay doi Team nhan xet thanh "ERO".
+4. Thay doi Ngay nhan xet thanh "2026-08-20".
+5. Nhan nut "Save".</t>
         </is>
       </c>
       <c r="J27" s="9" t="inlineStr">
         <is>
-          <t>Nhận xét được cập nhật thành công.
-Dữ liệu nhận xét được thay đổi với Team mới là "ERO" và ngày mới là "2026-08-20" trên giao diện.</t>
+          <t>Nhan xet duoc cap nhat successfully.
+Du lieu nhan xet duoc thay doi voi Team moi la "ERO" va ngay moi la "2026-08-20" tren interface.</t>
         </is>
       </c>
       <c r="K27" s="9" t="inlineStr"/>
@@ -3302,7 +3302,7 @@
       </c>
       <c r="N27" s="9" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F09, Rule 6.10</t>
+          <t>Related to M05-F09, Rule 6.10</t>
         </is>
       </c>
     </row>
@@ -3329,39 +3329,39 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Mở rộng/thu gọn danh sách học viên và hiển thị nhãn cảnh báo trong danh sách nhóm thực tập</t>
+          <t>Mo rong/thu gon danh sach student va display nhan cphoto bao trong danh sach internship group</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>Kiểm tra chức năng mở rộng/thu gọn (expand/collapse) của từng nhóm thực tập, điều hướng và hiển thị chính xác nhãn cảnh báo (Warning Badge).</t>
+          <t>Verify functionality for mo rong/thu gon (expand/collapse) cua tung internship group, dieu huong va display chinh xac nhan cphoto bao (Warning Badge).</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Người dùng đã đăng nhập với quyền Staff.
-Đang ở màn hình danh sách nhóm thực tập.
-Có nhóm thực tập "Nhóm Thực tập 2026" chứa 2 học viên chưa gán công ty.</t>
+          <t>User is logged in as Staff.
+Dang o man hinh danh sach internship group.
+Co internship group "Nhom Thuc tap 2026" chua 2 student chua gan company.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>GroupName="Nhóm Thực tập 2026"</t>
+          <t>GroupName="Nhom Thuc tap 2026"</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>1. Quan sát dòng hiển thị của nhóm thực tập "Nhóm Thực tập 2026".
-2. Kiểm tra xem có hiển thị nhãn cảnh báo học viên chưa gán hay không (ví dụ: "2 học viên chưa phân công" hoặc "2 Unassigned").
-3. Nhấp vào nút/biểu tượng mũi tên mở rộng (Expand) của nhóm thực tập này.
-4. Nhấp lại vào nút/biểu tượng thu gọn (Collapse) của nhóm thực tập.</t>
+          <t>1. Observe dong display cua internship group "Nhom Thuc tap 2026".
+2. Verify whether co display nhan cphoto bao student chua gan hay khong (e.g.: "2 student chua phan cong" hoac "2 Unassigned").
+3. Nhap vao nut/bieu tuong mui ten mo rong (Expand) cua internship group nay.
+4. Nhap lai vao nut/bieu tuong thu gon (Collapse) cua internship group.</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
         <is>
-          <t>Nhãn cảnh báo hiển thị chính xác số lượng học viên chưa gán (ví dụ: "⚠ 2 Unassigned" hoặc tương tự).
-Khi nhấn Mở rộng, danh sách học viên chi tiết của nhóm hiển thị ngay bên dưới.
-Khi nhấn Thu gọn, danh sách chi tiết được ẩn đi.</t>
+          <t>Nhan cphoto bao display chinh xac so luong student chua gan (e.g.: "⚠ 2 Unassigned" hoac tuong tu).
+Khi click Mo rong, danh sach student chi tiet cua group display ngay ben duoi.
+Khi click Thu gon, danh sach chi tiet duoc an di.</t>
         </is>
       </c>
       <c r="K28" s="4" t="inlineStr"/>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="N28" s="4" t="inlineStr">
         <is>
-          <t>Liên quan đến M05-F10, Rule 6.11</t>
+          <t>Related to M05-F10, Rule 6.11</t>
         </is>
       </c>
     </row>

</xml_diff>